<commit_message>
데이터 갱신 (풍고+엘로보드): 2026-09-03 14:55 UTC
</commit_message>
<xml_diff>
--- a/data/members.xlsx
+++ b/data/members.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X810"/>
+  <dimension ref="A1:W811"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -39207,10 +39207,25 @@
       <c r="C810" t="n">
         <v>773</v>
       </c>
-      <c r="E810" t="inlineStr"/>
-      <c r="F810" t="inlineStr"/>
-      <c r="G810" t="inlineStr"/>
-      <c r="H810" t="inlineStr"/>
+    </row>
+    <row r="811">
+      <c r="A811" t="inlineStr">
+        <is>
+          <t>미상(elo_763)</t>
+        </is>
+      </c>
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>elo_763</t>
+        </is>
+      </c>
+      <c r="C811" t="n">
+        <v>763</v>
+      </c>
+      <c r="E811" t="inlineStr"/>
+      <c r="F811" t="inlineStr"/>
+      <c r="G811" t="inlineStr"/>
+      <c r="H811" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -67292,7 +67307,6 @@
         <v/>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -69385,7 +69399,6 @@
         </is>
       </c>
     </row>
-    <row r="48"/>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>

</xml_diff>